<commit_message>
Update name row 75
</commit_message>
<xml_diff>
--- a/Datasets/NISQ_Bugs_Dataset.xlsx
+++ b/Datasets/NISQ_Bugs_Dataset.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10609"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10119"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://emckclac-my.sharepoint.com/personal/k20013502_kcl_ac_uk/Documents/NISQ_Taxonomy/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/avnerbensoussan/Downloads/A-Taxonomy-of-Real-Faults-in-Hybrid-Quantum-Classical-Architectures/Datasets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="8_{1A9542C3-800B-2C40-B740-B6D25EB42EE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A88C823F-929E-B240-8580-530271FB28A3}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EFC67D28-F3F3-AF4E-9ACA-E0E65381A539}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="42700" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="740" windowWidth="30240" windowHeight="18900" firstSheet="3" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="VQE" sheetId="1" r:id="rId1"/>
@@ -12620,7 +12620,7 @@
     </row>
     <row r="69" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
-        <v>408</v>
+        <v>36</v>
       </c>
       <c r="B69" s="44" t="s">
         <v>37</v>
@@ -15021,7 +15021,8 @@
   <dimension ref="A1:G134"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="10.83203125" customWidth="1"/>
+    <col min="1" max="1" width="77" customWidth="1"/>
+    <col min="2" max="2" width="46" customWidth="1"/>
     <col min="5" max="5" width="44.33203125" customWidth="1"/>
     <col min="6" max="6" width="66.5" customWidth="1"/>
     <col min="7" max="7" width="255.6640625" customWidth="1"/>
@@ -15282,7 +15283,7 @@
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>408</v>
+        <v>36</v>
       </c>
       <c r="B12" s="44" t="s">
         <v>37</v>
@@ -19327,7 +19328,7 @@
     </row>
     <row r="14" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>408</v>
+        <v>36</v>
       </c>
       <c r="B14" s="44" t="s">
         <v>37</v>

</xml_diff>